<commit_message>
auto: solar data update 2026-07-20
</commit_message>
<xml_diff>
--- a/log.xlsx
+++ b/log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1921"/>
+  <dimension ref="A1:L1945"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -81598,6 +81598,1014 @@
         <v>10.7</v>
       </c>
     </row>
+    <row r="1922">
+      <c r="A1922" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B1922" t="inlineStr">
+        <is>
+          <t>0시</t>
+        </is>
+      </c>
+      <c r="C1922" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1922" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1922" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1922" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="G1922" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="H1922" t="n">
+        <v>0</v>
+      </c>
+      <c r="I1922" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1922" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1922" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="L1922" t="n">
+        <v>13.5</v>
+      </c>
+    </row>
+    <row r="1923">
+      <c r="A1923" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B1923" t="inlineStr">
+        <is>
+          <t>1시</t>
+        </is>
+      </c>
+      <c r="C1923" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1923" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1923" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1923" t="n">
+        <v>24.1</v>
+      </c>
+      <c r="G1923" t="n">
+        <v>11.9</v>
+      </c>
+      <c r="H1923" t="n">
+        <v>0</v>
+      </c>
+      <c r="I1923" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1923" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1923" t="n">
+        <v>24.1</v>
+      </c>
+      <c r="L1923" t="n">
+        <v>11.9</v>
+      </c>
+    </row>
+    <row r="1924">
+      <c r="A1924" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B1924" t="inlineStr">
+        <is>
+          <t>2시</t>
+        </is>
+      </c>
+      <c r="C1924" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1924" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1924" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1924" t="n">
+        <v>24.1</v>
+      </c>
+      <c r="G1924" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="H1924" t="n">
+        <v>0</v>
+      </c>
+      <c r="I1924" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1924" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1924" t="n">
+        <v>24.1</v>
+      </c>
+      <c r="L1924" t="n">
+        <v>6.1</v>
+      </c>
+    </row>
+    <row r="1925">
+      <c r="A1925" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B1925" t="inlineStr">
+        <is>
+          <t>3시</t>
+        </is>
+      </c>
+      <c r="C1925" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1925" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1925" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1925" t="n">
+        <v>24.2</v>
+      </c>
+      <c r="G1925" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="H1925" t="n">
+        <v>0</v>
+      </c>
+      <c r="I1925" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1925" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1925" t="n">
+        <v>24.2</v>
+      </c>
+      <c r="L1925" t="n">
+        <v>7.3</v>
+      </c>
+    </row>
+    <row r="1926">
+      <c r="A1926" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B1926" t="inlineStr">
+        <is>
+          <t>4시</t>
+        </is>
+      </c>
+      <c r="C1926" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1926" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1926" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1926" t="n">
+        <v>23.7</v>
+      </c>
+      <c r="G1926" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="H1926" t="n">
+        <v>0</v>
+      </c>
+      <c r="I1926" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1926" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1926" t="n">
+        <v>23.7</v>
+      </c>
+      <c r="L1926" t="n">
+        <v>7.6</v>
+      </c>
+    </row>
+    <row r="1927">
+      <c r="A1927" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B1927" t="inlineStr">
+        <is>
+          <t>5시</t>
+        </is>
+      </c>
+      <c r="C1927" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1927" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1927" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1927" t="n">
+        <v>23.4</v>
+      </c>
+      <c r="G1927" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="H1927" t="n">
+        <v>0</v>
+      </c>
+      <c r="I1927" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1927" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1927" t="n">
+        <v>23.4</v>
+      </c>
+      <c r="L1927" t="n">
+        <v>8.800000000000001</v>
+      </c>
+    </row>
+    <row r="1928">
+      <c r="A1928" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B1928" t="inlineStr">
+        <is>
+          <t>6시</t>
+        </is>
+      </c>
+      <c r="C1928" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="D1928" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="E1928" t="n">
+        <v>4</v>
+      </c>
+      <c r="F1928" t="n">
+        <v>23.4</v>
+      </c>
+      <c r="G1928" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="H1928" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="I1928" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="J1928" t="n">
+        <v>4</v>
+      </c>
+      <c r="K1928" t="n">
+        <v>23.4</v>
+      </c>
+      <c r="L1928" t="n">
+        <v>10.2</v>
+      </c>
+    </row>
+    <row r="1929">
+      <c r="A1929" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B1929" t="inlineStr">
+        <is>
+          <t>7시</t>
+        </is>
+      </c>
+      <c r="C1929" t="n">
+        <v>3.26</v>
+      </c>
+      <c r="D1929" t="n">
+        <v>3.59</v>
+      </c>
+      <c r="E1929" t="n">
+        <v>40</v>
+      </c>
+      <c r="F1929" t="n">
+        <v>23.8</v>
+      </c>
+      <c r="G1929" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="H1929" t="n">
+        <v>3.26</v>
+      </c>
+      <c r="I1929" t="n">
+        <v>3.59</v>
+      </c>
+      <c r="J1929" t="n">
+        <v>40</v>
+      </c>
+      <c r="K1929" t="n">
+        <v>23.8</v>
+      </c>
+      <c r="L1929" t="n">
+        <v>8.5</v>
+      </c>
+    </row>
+    <row r="1930">
+      <c r="A1930" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B1930" t="inlineStr">
+        <is>
+          <t>8시</t>
+        </is>
+      </c>
+      <c r="C1930" t="n">
+        <v>7.37</v>
+      </c>
+      <c r="D1930" t="n">
+        <v>10.96</v>
+      </c>
+      <c r="E1930" t="n">
+        <v>91</v>
+      </c>
+      <c r="F1930" t="n">
+        <v>23.9</v>
+      </c>
+      <c r="G1930" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="H1930" t="n">
+        <v>7.37</v>
+      </c>
+      <c r="I1930" t="n">
+        <v>10.96</v>
+      </c>
+      <c r="J1930" t="n">
+        <v>91</v>
+      </c>
+      <c r="K1930" t="n">
+        <v>23.9</v>
+      </c>
+      <c r="L1930" t="n">
+        <v>3.4</v>
+      </c>
+    </row>
+    <row r="1931">
+      <c r="A1931" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B1931" t="inlineStr">
+        <is>
+          <t>9시</t>
+        </is>
+      </c>
+      <c r="C1931" t="n">
+        <v>17.49</v>
+      </c>
+      <c r="D1931" t="n">
+        <v>28.45</v>
+      </c>
+      <c r="E1931" t="n">
+        <v>220</v>
+      </c>
+      <c r="F1931" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="G1931" t="n">
+        <v>7</v>
+      </c>
+      <c r="H1931" t="n">
+        <v>17.49</v>
+      </c>
+      <c r="I1931" t="n">
+        <v>28.45</v>
+      </c>
+      <c r="J1931" t="n">
+        <v>220</v>
+      </c>
+      <c r="K1931" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="L1931" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="1932">
+      <c r="A1932" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B1932" t="inlineStr">
+        <is>
+          <t>10시</t>
+        </is>
+      </c>
+      <c r="C1932" t="n">
+        <v>20.38</v>
+      </c>
+      <c r="D1932" t="n">
+        <v>48.83</v>
+      </c>
+      <c r="E1932" t="n">
+        <v>258</v>
+      </c>
+      <c r="F1932" t="n">
+        <v>24.9</v>
+      </c>
+      <c r="G1932" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="H1932" t="n">
+        <v>20.38</v>
+      </c>
+      <c r="I1932" t="n">
+        <v>48.83</v>
+      </c>
+      <c r="J1932" t="n">
+        <v>258</v>
+      </c>
+      <c r="K1932" t="n">
+        <v>24.9</v>
+      </c>
+      <c r="L1932" t="n">
+        <v>8.6</v>
+      </c>
+    </row>
+    <row r="1933">
+      <c r="A1933" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B1933" t="inlineStr">
+        <is>
+          <t>11시</t>
+        </is>
+      </c>
+      <c r="C1933" t="n">
+        <v>24.62</v>
+      </c>
+      <c r="D1933" t="n">
+        <v>73.45</v>
+      </c>
+      <c r="E1933" t="n">
+        <v>315</v>
+      </c>
+      <c r="F1933" t="n">
+        <v>25.7</v>
+      </c>
+      <c r="G1933" t="n">
+        <v>13.7</v>
+      </c>
+      <c r="H1933" t="n">
+        <v>24.62</v>
+      </c>
+      <c r="I1933" t="n">
+        <v>73.45</v>
+      </c>
+      <c r="J1933" t="n">
+        <v>315</v>
+      </c>
+      <c r="K1933" t="n">
+        <v>25.7</v>
+      </c>
+      <c r="L1933" t="n">
+        <v>13.7</v>
+      </c>
+    </row>
+    <row r="1934">
+      <c r="A1934" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B1934" t="inlineStr">
+        <is>
+          <t>12시</t>
+        </is>
+      </c>
+      <c r="C1934" t="n">
+        <v>37.8</v>
+      </c>
+      <c r="D1934" t="n">
+        <v>111.25</v>
+      </c>
+      <c r="E1934" t="n">
+        <v>498</v>
+      </c>
+      <c r="F1934" t="n">
+        <v>26.9</v>
+      </c>
+      <c r="G1934" t="n">
+        <v>14.8</v>
+      </c>
+      <c r="H1934" t="n">
+        <v>37.8</v>
+      </c>
+      <c r="I1934" t="n">
+        <v>111.25</v>
+      </c>
+      <c r="J1934" t="n">
+        <v>498</v>
+      </c>
+      <c r="K1934" t="n">
+        <v>26.9</v>
+      </c>
+      <c r="L1934" t="n">
+        <v>14.8</v>
+      </c>
+    </row>
+    <row r="1935">
+      <c r="A1935" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B1935" t="inlineStr">
+        <is>
+          <t>13시</t>
+        </is>
+      </c>
+      <c r="C1935" t="n">
+        <v>52.33</v>
+      </c>
+      <c r="D1935" t="n">
+        <v>163.58</v>
+      </c>
+      <c r="E1935" t="n">
+        <v>716</v>
+      </c>
+      <c r="F1935" t="n">
+        <v>28.7</v>
+      </c>
+      <c r="G1935" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="H1935" t="n">
+        <v>52.33</v>
+      </c>
+      <c r="I1935" t="n">
+        <v>163.58</v>
+      </c>
+      <c r="J1935" t="n">
+        <v>716</v>
+      </c>
+      <c r="K1935" t="n">
+        <v>28.7</v>
+      </c>
+      <c r="L1935" t="n">
+        <v>13.4</v>
+      </c>
+    </row>
+    <row r="1936">
+      <c r="A1936" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B1936" t="inlineStr">
+        <is>
+          <t>14시</t>
+        </is>
+      </c>
+      <c r="C1936" t="n">
+        <v>47.77</v>
+      </c>
+      <c r="D1936" t="n">
+        <v>211.35</v>
+      </c>
+      <c r="E1936" t="n">
+        <v>649</v>
+      </c>
+      <c r="F1936" t="n">
+        <v>29.2</v>
+      </c>
+      <c r="G1936" t="n">
+        <v>13</v>
+      </c>
+      <c r="H1936" t="n">
+        <v>47.77</v>
+      </c>
+      <c r="I1936" t="n">
+        <v>211.35</v>
+      </c>
+      <c r="J1936" t="n">
+        <v>649</v>
+      </c>
+      <c r="K1936" t="n">
+        <v>29.2</v>
+      </c>
+      <c r="L1936" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="1937">
+      <c r="A1937" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B1937" t="inlineStr">
+        <is>
+          <t>15시</t>
+        </is>
+      </c>
+      <c r="C1937" t="n">
+        <v>49.37</v>
+      </c>
+      <c r="D1937" t="n">
+        <v>260.72</v>
+      </c>
+      <c r="E1937" t="n">
+        <v>672</v>
+      </c>
+      <c r="F1937" t="n">
+        <v>28.9</v>
+      </c>
+      <c r="G1937" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="H1937" t="n">
+        <v>49.37</v>
+      </c>
+      <c r="I1937" t="n">
+        <v>260.72</v>
+      </c>
+      <c r="J1937" t="n">
+        <v>672</v>
+      </c>
+      <c r="K1937" t="n">
+        <v>28.9</v>
+      </c>
+      <c r="L1937" t="n">
+        <v>11.5</v>
+      </c>
+    </row>
+    <row r="1938">
+      <c r="A1938" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B1938" t="inlineStr">
+        <is>
+          <t>16시</t>
+        </is>
+      </c>
+      <c r="C1938" t="n">
+        <v>38.05</v>
+      </c>
+      <c r="D1938" t="n">
+        <v>298.77</v>
+      </c>
+      <c r="E1938" t="n">
+        <v>507</v>
+      </c>
+      <c r="F1938" t="n">
+        <v>29.2</v>
+      </c>
+      <c r="G1938" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="H1938" t="n">
+        <v>38.05</v>
+      </c>
+      <c r="I1938" t="n">
+        <v>298.77</v>
+      </c>
+      <c r="J1938" t="n">
+        <v>507</v>
+      </c>
+      <c r="K1938" t="n">
+        <v>29.2</v>
+      </c>
+      <c r="L1938" t="n">
+        <v>11.4</v>
+      </c>
+    </row>
+    <row r="1939">
+      <c r="A1939" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B1939" t="inlineStr">
+        <is>
+          <t>17시</t>
+        </is>
+      </c>
+      <c r="C1939" t="n">
+        <v>29.67</v>
+      </c>
+      <c r="D1939" t="n">
+        <v>328.44</v>
+      </c>
+      <c r="E1939" t="n">
+        <v>389</v>
+      </c>
+      <c r="F1939" t="n">
+        <v>29.2</v>
+      </c>
+      <c r="G1939" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="H1939" t="n">
+        <v>29.67</v>
+      </c>
+      <c r="I1939" t="n">
+        <v>328.44</v>
+      </c>
+      <c r="J1939" t="n">
+        <v>389</v>
+      </c>
+      <c r="K1939" t="n">
+        <v>29.2</v>
+      </c>
+      <c r="L1939" t="n">
+        <v>11.2</v>
+      </c>
+    </row>
+    <row r="1940">
+      <c r="A1940" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B1940" t="inlineStr">
+        <is>
+          <t>18시</t>
+        </is>
+      </c>
+      <c r="C1940" t="n">
+        <v>20.6</v>
+      </c>
+      <c r="D1940" t="n">
+        <v>349.04</v>
+      </c>
+      <c r="E1940" t="n">
+        <v>265</v>
+      </c>
+      <c r="F1940" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="G1940" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="H1940" t="n">
+        <v>20.6</v>
+      </c>
+      <c r="I1940" t="n">
+        <v>349.04</v>
+      </c>
+      <c r="J1940" t="n">
+        <v>265</v>
+      </c>
+      <c r="K1940" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="L1940" t="n">
+        <v>10.5</v>
+      </c>
+    </row>
+    <row r="1941">
+      <c r="A1941" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B1941" t="inlineStr">
+        <is>
+          <t>19시</t>
+        </is>
+      </c>
+      <c r="C1941" t="n">
+        <v>8.220000000000001</v>
+      </c>
+      <c r="D1941" t="n">
+        <v>357.26</v>
+      </c>
+      <c r="E1941" t="n">
+        <v>103</v>
+      </c>
+      <c r="F1941" t="n">
+        <v>27.3</v>
+      </c>
+      <c r="G1941" t="n">
+        <v>9.699999999999999</v>
+      </c>
+      <c r="H1941" t="n">
+        <v>8.220000000000001</v>
+      </c>
+      <c r="I1941" t="n">
+        <v>357.26</v>
+      </c>
+      <c r="J1941" t="n">
+        <v>103</v>
+      </c>
+      <c r="K1941" t="n">
+        <v>27.3</v>
+      </c>
+      <c r="L1941" t="n">
+        <v>9.699999999999999</v>
+      </c>
+    </row>
+    <row r="1942">
+      <c r="A1942" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B1942" t="inlineStr">
+        <is>
+          <t>20시</t>
+        </is>
+      </c>
+      <c r="C1942" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="D1942" t="n">
+        <v>358.31</v>
+      </c>
+      <c r="E1942" t="n">
+        <v>13</v>
+      </c>
+      <c r="F1942" t="n">
+        <v>26.1</v>
+      </c>
+      <c r="G1942" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="H1942" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="I1942" t="n">
+        <v>358.31</v>
+      </c>
+      <c r="J1942" t="n">
+        <v>13</v>
+      </c>
+      <c r="K1942" t="n">
+        <v>26.1</v>
+      </c>
+      <c r="L1942" t="n">
+        <v>6.4</v>
+      </c>
+    </row>
+    <row r="1943">
+      <c r="A1943" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B1943" t="inlineStr">
+        <is>
+          <t>21시</t>
+        </is>
+      </c>
+      <c r="C1943" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1943" t="n">
+        <v>358.31</v>
+      </c>
+      <c r="E1943" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1943" t="n">
+        <v>25.3</v>
+      </c>
+      <c r="G1943" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="H1943" t="n">
+        <v>0</v>
+      </c>
+      <c r="I1943" t="n">
+        <v>358.31</v>
+      </c>
+      <c r="J1943" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1943" t="n">
+        <v>25.3</v>
+      </c>
+      <c r="L1943" t="n">
+        <v>6.3</v>
+      </c>
+    </row>
+    <row r="1944">
+      <c r="A1944" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B1944" t="inlineStr">
+        <is>
+          <t>22시</t>
+        </is>
+      </c>
+      <c r="C1944" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1944" t="n">
+        <v>358.31</v>
+      </c>
+      <c r="E1944" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1944" t="n">
+        <v>24.8</v>
+      </c>
+      <c r="G1944" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="H1944" t="n">
+        <v>0</v>
+      </c>
+      <c r="I1944" t="n">
+        <v>358.31</v>
+      </c>
+      <c r="J1944" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1944" t="n">
+        <v>24.8</v>
+      </c>
+      <c r="L1944" t="n">
+        <v>6.8</v>
+      </c>
+    </row>
+    <row r="1945">
+      <c r="A1945" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B1945" t="inlineStr">
+        <is>
+          <t>23시</t>
+        </is>
+      </c>
+      <c r="C1945" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1945" t="n">
+        <v>358.31</v>
+      </c>
+      <c r="E1945" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1945" t="n">
+        <v>24.3</v>
+      </c>
+      <c r="G1945" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="H1945" t="n">
+        <v>0</v>
+      </c>
+      <c r="I1945" t="n">
+        <v>358.31</v>
+      </c>
+      <c r="J1945" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1945" t="n">
+        <v>24.3</v>
+      </c>
+      <c r="L1945" t="n">
+        <v>7.2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto: solar data update 2026-07-21
</commit_message>
<xml_diff>
--- a/log.xlsx
+++ b/log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1945"/>
+  <dimension ref="A1:L1969"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -82606,6 +82606,1014 @@
         <v>7.2</v>
       </c>
     </row>
+    <row r="1946">
+      <c r="A1946" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B1946" t="inlineStr">
+        <is>
+          <t>0시</t>
+        </is>
+      </c>
+      <c r="C1946" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1946" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1946" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1946" t="n">
+        <v>23.6</v>
+      </c>
+      <c r="G1946" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="H1946" t="n">
+        <v>0</v>
+      </c>
+      <c r="I1946" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1946" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1946" t="n">
+        <v>23.6</v>
+      </c>
+      <c r="L1946" t="n">
+        <v>10.4</v>
+      </c>
+    </row>
+    <row r="1947">
+      <c r="A1947" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B1947" t="inlineStr">
+        <is>
+          <t>1시</t>
+        </is>
+      </c>
+      <c r="C1947" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1947" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1947" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1947" t="n">
+        <v>23</v>
+      </c>
+      <c r="G1947" t="n">
+        <v>5</v>
+      </c>
+      <c r="H1947" t="n">
+        <v>0</v>
+      </c>
+      <c r="I1947" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1947" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1947" t="n">
+        <v>23</v>
+      </c>
+      <c r="L1947" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1948">
+      <c r="A1948" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B1948" t="inlineStr">
+        <is>
+          <t>2시</t>
+        </is>
+      </c>
+      <c r="C1948" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1948" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1948" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1948" t="n">
+        <v>22.9</v>
+      </c>
+      <c r="G1948" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H1948" t="n">
+        <v>0</v>
+      </c>
+      <c r="I1948" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1948" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1948" t="n">
+        <v>22.9</v>
+      </c>
+      <c r="L1948" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="1949">
+      <c r="A1949" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B1949" t="inlineStr">
+        <is>
+          <t>3시</t>
+        </is>
+      </c>
+      <c r="C1949" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1949" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1949" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1949" t="n">
+        <v>22.6</v>
+      </c>
+      <c r="G1949" t="n">
+        <v>3</v>
+      </c>
+      <c r="H1949" t="n">
+        <v>0</v>
+      </c>
+      <c r="I1949" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1949" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1949" t="n">
+        <v>22.6</v>
+      </c>
+      <c r="L1949" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1950">
+      <c r="A1950" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B1950" t="inlineStr">
+        <is>
+          <t>4시</t>
+        </is>
+      </c>
+      <c r="C1950" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1950" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1950" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1950" t="n">
+        <v>22.9</v>
+      </c>
+      <c r="G1950" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="H1950" t="n">
+        <v>0</v>
+      </c>
+      <c r="I1950" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1950" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1950" t="n">
+        <v>22.9</v>
+      </c>
+      <c r="L1950" t="n">
+        <v>7.6</v>
+      </c>
+    </row>
+    <row r="1951">
+      <c r="A1951" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B1951" t="inlineStr">
+        <is>
+          <t>5시</t>
+        </is>
+      </c>
+      <c r="C1951" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1951" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1951" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1951" t="n">
+        <v>22.3</v>
+      </c>
+      <c r="G1951" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="H1951" t="n">
+        <v>0</v>
+      </c>
+      <c r="I1951" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1951" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1951" t="n">
+        <v>22.3</v>
+      </c>
+      <c r="L1951" t="n">
+        <v>9.199999999999999</v>
+      </c>
+    </row>
+    <row r="1952">
+      <c r="A1952" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B1952" t="inlineStr">
+        <is>
+          <t>6시</t>
+        </is>
+      </c>
+      <c r="C1952" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="D1952" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="E1952" t="n">
+        <v>7</v>
+      </c>
+      <c r="F1952" t="n">
+        <v>22.1</v>
+      </c>
+      <c r="G1952" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="H1952" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="I1952" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="J1952" t="n">
+        <v>7</v>
+      </c>
+      <c r="K1952" t="n">
+        <v>22.1</v>
+      </c>
+      <c r="L1952" t="n">
+        <v>8.1</v>
+      </c>
+    </row>
+    <row r="1953">
+      <c r="A1953" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B1953" t="inlineStr">
+        <is>
+          <t>7시</t>
+        </is>
+      </c>
+      <c r="C1953" t="n">
+        <v>6.84</v>
+      </c>
+      <c r="D1953" t="n">
+        <v>7.41</v>
+      </c>
+      <c r="E1953" t="n">
+        <v>84</v>
+      </c>
+      <c r="F1953" t="n">
+        <v>23</v>
+      </c>
+      <c r="G1953" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="H1953" t="n">
+        <v>6.84</v>
+      </c>
+      <c r="I1953" t="n">
+        <v>7.41</v>
+      </c>
+      <c r="J1953" t="n">
+        <v>84</v>
+      </c>
+      <c r="K1953" t="n">
+        <v>23</v>
+      </c>
+      <c r="L1953" t="n">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="1954">
+      <c r="A1954" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B1954" t="inlineStr">
+        <is>
+          <t>8시</t>
+        </is>
+      </c>
+      <c r="C1954" t="n">
+        <v>11.68</v>
+      </c>
+      <c r="D1954" t="n">
+        <v>19.09</v>
+      </c>
+      <c r="E1954" t="n">
+        <v>145</v>
+      </c>
+      <c r="F1954" t="n">
+        <v>23.6</v>
+      </c>
+      <c r="G1954" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="H1954" t="n">
+        <v>11.68</v>
+      </c>
+      <c r="I1954" t="n">
+        <v>19.09</v>
+      </c>
+      <c r="J1954" t="n">
+        <v>145</v>
+      </c>
+      <c r="K1954" t="n">
+        <v>23.6</v>
+      </c>
+      <c r="L1954" t="n">
+        <v>3.2</v>
+      </c>
+    </row>
+    <row r="1955">
+      <c r="A1955" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B1955" t="inlineStr">
+        <is>
+          <t>9시</t>
+        </is>
+      </c>
+      <c r="C1955" t="n">
+        <v>29.82</v>
+      </c>
+      <c r="D1955" t="n">
+        <v>48.91</v>
+      </c>
+      <c r="E1955" t="n">
+        <v>385</v>
+      </c>
+      <c r="F1955" t="n">
+        <v>25.7</v>
+      </c>
+      <c r="G1955" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="H1955" t="n">
+        <v>29.82</v>
+      </c>
+      <c r="I1955" t="n">
+        <v>48.91</v>
+      </c>
+      <c r="J1955" t="n">
+        <v>385</v>
+      </c>
+      <c r="K1955" t="n">
+        <v>25.7</v>
+      </c>
+      <c r="L1955" t="n">
+        <v>12.8</v>
+      </c>
+    </row>
+    <row r="1956">
+      <c r="A1956" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B1956" t="inlineStr">
+        <is>
+          <t>10시</t>
+        </is>
+      </c>
+      <c r="C1956" t="n">
+        <v>44.11</v>
+      </c>
+      <c r="D1956" t="n">
+        <v>93.02</v>
+      </c>
+      <c r="E1956" t="n">
+        <v>588</v>
+      </c>
+      <c r="F1956" t="n">
+        <v>26.8</v>
+      </c>
+      <c r="G1956" t="n">
+        <v>15.7</v>
+      </c>
+      <c r="H1956" t="n">
+        <v>44.11</v>
+      </c>
+      <c r="I1956" t="n">
+        <v>93.02</v>
+      </c>
+      <c r="J1956" t="n">
+        <v>588</v>
+      </c>
+      <c r="K1956" t="n">
+        <v>26.8</v>
+      </c>
+      <c r="L1956" t="n">
+        <v>15.7</v>
+      </c>
+    </row>
+    <row r="1957">
+      <c r="A1957" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B1957" t="inlineStr">
+        <is>
+          <t>11시</t>
+        </is>
+      </c>
+      <c r="C1957" t="n">
+        <v>57.17</v>
+      </c>
+      <c r="D1957" t="n">
+        <v>150.19</v>
+      </c>
+      <c r="E1957" t="n">
+        <v>790</v>
+      </c>
+      <c r="F1957" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="G1957" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="H1957" t="n">
+        <v>57.17</v>
+      </c>
+      <c r="I1957" t="n">
+        <v>150.19</v>
+      </c>
+      <c r="J1957" t="n">
+        <v>790</v>
+      </c>
+      <c r="K1957" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="L1957" t="n">
+        <v>16.9</v>
+      </c>
+    </row>
+    <row r="1958">
+      <c r="A1958" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B1958" t="inlineStr">
+        <is>
+          <t>12시</t>
+        </is>
+      </c>
+      <c r="C1958" t="n">
+        <v>60.53</v>
+      </c>
+      <c r="D1958" t="n">
+        <v>210.72</v>
+      </c>
+      <c r="E1958" t="n">
+        <v>847</v>
+      </c>
+      <c r="F1958" t="n">
+        <v>29.6</v>
+      </c>
+      <c r="G1958" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="H1958" t="n">
+        <v>60.53</v>
+      </c>
+      <c r="I1958" t="n">
+        <v>210.72</v>
+      </c>
+      <c r="J1958" t="n">
+        <v>847</v>
+      </c>
+      <c r="K1958" t="n">
+        <v>29.6</v>
+      </c>
+      <c r="L1958" t="n">
+        <v>15.5</v>
+      </c>
+    </row>
+    <row r="1959">
+      <c r="A1959" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B1959" t="inlineStr">
+        <is>
+          <t>13시</t>
+        </is>
+      </c>
+      <c r="C1959" t="n">
+        <v>61.85</v>
+      </c>
+      <c r="D1959" t="n">
+        <v>272.57</v>
+      </c>
+      <c r="E1959" t="n">
+        <v>869</v>
+      </c>
+      <c r="F1959" t="n">
+        <v>29.8</v>
+      </c>
+      <c r="G1959" t="n">
+        <v>16.4</v>
+      </c>
+      <c r="H1959" t="n">
+        <v>61.85</v>
+      </c>
+      <c r="I1959" t="n">
+        <v>272.57</v>
+      </c>
+      <c r="J1959" t="n">
+        <v>869</v>
+      </c>
+      <c r="K1959" t="n">
+        <v>29.8</v>
+      </c>
+      <c r="L1959" t="n">
+        <v>16.4</v>
+      </c>
+    </row>
+    <row r="1960">
+      <c r="A1960" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B1960" t="inlineStr">
+        <is>
+          <t>14시</t>
+        </is>
+      </c>
+      <c r="C1960" t="n">
+        <v>61.85</v>
+      </c>
+      <c r="D1960" t="n">
+        <v>334.42</v>
+      </c>
+      <c r="E1960" t="n">
+        <v>870</v>
+      </c>
+      <c r="F1960" t="n">
+        <v>30</v>
+      </c>
+      <c r="G1960" t="n">
+        <v>17.4</v>
+      </c>
+      <c r="H1960" t="n">
+        <v>61.85</v>
+      </c>
+      <c r="I1960" t="n">
+        <v>334.42</v>
+      </c>
+      <c r="J1960" t="n">
+        <v>870</v>
+      </c>
+      <c r="K1960" t="n">
+        <v>30</v>
+      </c>
+      <c r="L1960" t="n">
+        <v>17.4</v>
+      </c>
+    </row>
+    <row r="1961">
+      <c r="A1961" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B1961" t="inlineStr">
+        <is>
+          <t>15시</t>
+        </is>
+      </c>
+      <c r="C1961" t="n">
+        <v>53.91</v>
+      </c>
+      <c r="D1961" t="n">
+        <v>388.33</v>
+      </c>
+      <c r="E1961" t="n">
+        <v>745</v>
+      </c>
+      <c r="F1961" t="n">
+        <v>30</v>
+      </c>
+      <c r="G1961" t="n">
+        <v>19.3</v>
+      </c>
+      <c r="H1961" t="n">
+        <v>53.91</v>
+      </c>
+      <c r="I1961" t="n">
+        <v>388.33</v>
+      </c>
+      <c r="J1961" t="n">
+        <v>745</v>
+      </c>
+      <c r="K1961" t="n">
+        <v>30</v>
+      </c>
+      <c r="L1961" t="n">
+        <v>19.3</v>
+      </c>
+    </row>
+    <row r="1962">
+      <c r="A1962" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B1962" t="inlineStr">
+        <is>
+          <t>16시</t>
+        </is>
+      </c>
+      <c r="C1962" t="n">
+        <v>47.95</v>
+      </c>
+      <c r="D1962" t="n">
+        <v>436.28</v>
+      </c>
+      <c r="E1962" t="n">
+        <v>652</v>
+      </c>
+      <c r="F1962" t="n">
+        <v>29.3</v>
+      </c>
+      <c r="G1962" t="n">
+        <v>21</v>
+      </c>
+      <c r="H1962" t="n">
+        <v>47.95</v>
+      </c>
+      <c r="I1962" t="n">
+        <v>436.28</v>
+      </c>
+      <c r="J1962" t="n">
+        <v>652</v>
+      </c>
+      <c r="K1962" t="n">
+        <v>29.3</v>
+      </c>
+      <c r="L1962" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="1963">
+      <c r="A1963" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B1963" t="inlineStr">
+        <is>
+          <t>17시</t>
+        </is>
+      </c>
+      <c r="C1963" t="n">
+        <v>36.94</v>
+      </c>
+      <c r="D1963" t="n">
+        <v>473.22</v>
+      </c>
+      <c r="E1963" t="n">
+        <v>490</v>
+      </c>
+      <c r="F1963" t="n">
+        <v>28.7</v>
+      </c>
+      <c r="G1963" t="n">
+        <v>19.3</v>
+      </c>
+      <c r="H1963" t="n">
+        <v>36.94</v>
+      </c>
+      <c r="I1963" t="n">
+        <v>473.22</v>
+      </c>
+      <c r="J1963" t="n">
+        <v>490</v>
+      </c>
+      <c r="K1963" t="n">
+        <v>28.7</v>
+      </c>
+      <c r="L1963" t="n">
+        <v>19.3</v>
+      </c>
+    </row>
+    <row r="1964">
+      <c r="A1964" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B1964" t="inlineStr">
+        <is>
+          <t>18시</t>
+        </is>
+      </c>
+      <c r="C1964" t="n">
+        <v>24.09</v>
+      </c>
+      <c r="D1964" t="n">
+        <v>497.31</v>
+      </c>
+      <c r="E1964" t="n">
+        <v>311</v>
+      </c>
+      <c r="F1964" t="n">
+        <v>28</v>
+      </c>
+      <c r="G1964" t="n">
+        <v>17.2</v>
+      </c>
+      <c r="H1964" t="n">
+        <v>24.09</v>
+      </c>
+      <c r="I1964" t="n">
+        <v>497.31</v>
+      </c>
+      <c r="J1964" t="n">
+        <v>311</v>
+      </c>
+      <c r="K1964" t="n">
+        <v>28</v>
+      </c>
+      <c r="L1964" t="n">
+        <v>17.2</v>
+      </c>
+    </row>
+    <row r="1965">
+      <c r="A1965" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B1965" t="inlineStr">
+        <is>
+          <t>19시</t>
+        </is>
+      </c>
+      <c r="C1965" t="n">
+        <v>10.73</v>
+      </c>
+      <c r="D1965" t="n">
+        <v>508.04</v>
+      </c>
+      <c r="E1965" t="n">
+        <v>135</v>
+      </c>
+      <c r="F1965" t="n">
+        <v>27.2</v>
+      </c>
+      <c r="G1965" t="n">
+        <v>13</v>
+      </c>
+      <c r="H1965" t="n">
+        <v>10.73</v>
+      </c>
+      <c r="I1965" t="n">
+        <v>508.04</v>
+      </c>
+      <c r="J1965" t="n">
+        <v>135</v>
+      </c>
+      <c r="K1965" t="n">
+        <v>27.2</v>
+      </c>
+      <c r="L1965" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="1966">
+      <c r="A1966" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B1966" t="inlineStr">
+        <is>
+          <t>20시</t>
+        </is>
+      </c>
+      <c r="C1966" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="D1966" t="n">
+        <v>509.26</v>
+      </c>
+      <c r="E1966" t="n">
+        <v>15</v>
+      </c>
+      <c r="F1966" t="n">
+        <v>26</v>
+      </c>
+      <c r="G1966" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="H1966" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="I1966" t="n">
+        <v>509.26</v>
+      </c>
+      <c r="J1966" t="n">
+        <v>15</v>
+      </c>
+      <c r="K1966" t="n">
+        <v>26</v>
+      </c>
+      <c r="L1966" t="n">
+        <v>11.2</v>
+      </c>
+    </row>
+    <row r="1967">
+      <c r="A1967" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B1967" t="inlineStr">
+        <is>
+          <t>21시</t>
+        </is>
+      </c>
+      <c r="C1967" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1967" t="n">
+        <v>509.26</v>
+      </c>
+      <c r="E1967" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1967" t="n">
+        <v>25.4</v>
+      </c>
+      <c r="G1967" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="H1967" t="n">
+        <v>0</v>
+      </c>
+      <c r="I1967" t="n">
+        <v>509.26</v>
+      </c>
+      <c r="J1967" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1967" t="n">
+        <v>25.4</v>
+      </c>
+      <c r="L1967" t="n">
+        <v>10.8</v>
+      </c>
+    </row>
+    <row r="1968">
+      <c r="A1968" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B1968" t="inlineStr">
+        <is>
+          <t>22시</t>
+        </is>
+      </c>
+      <c r="C1968" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1968" t="n">
+        <v>509.26</v>
+      </c>
+      <c r="E1968" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1968" t="n">
+        <v>25</v>
+      </c>
+      <c r="G1968" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="H1968" t="n">
+        <v>0</v>
+      </c>
+      <c r="I1968" t="n">
+        <v>509.26</v>
+      </c>
+      <c r="J1968" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1968" t="n">
+        <v>25</v>
+      </c>
+      <c r="L1968" t="n">
+        <v>8.1</v>
+      </c>
+    </row>
+    <row r="1969">
+      <c r="A1969" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B1969" t="inlineStr">
+        <is>
+          <t>23시</t>
+        </is>
+      </c>
+      <c r="C1969" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1969" t="n">
+        <v>509.26</v>
+      </c>
+      <c r="E1969" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1969" t="n">
+        <v>24.6</v>
+      </c>
+      <c r="G1969" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="H1969" t="n">
+        <v>0</v>
+      </c>
+      <c r="I1969" t="n">
+        <v>509.26</v>
+      </c>
+      <c r="J1969" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1969" t="n">
+        <v>24.6</v>
+      </c>
+      <c r="L1969" t="n">
+        <v>7.2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto: solar data update 2026-07-31
</commit_message>
<xml_diff>
--- a/log.xlsx
+++ b/log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1969"/>
+  <dimension ref="A1:L1993"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -83614,6 +83614,1014 @@
         <v>7.2</v>
       </c>
     </row>
+    <row r="1970">
+      <c r="A1970" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B1970" t="inlineStr">
+        <is>
+          <t>0시</t>
+        </is>
+      </c>
+      <c r="C1970" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1970" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1970" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1970" t="n">
+        <v>26.6</v>
+      </c>
+      <c r="G1970" t="n">
+        <v>6</v>
+      </c>
+      <c r="H1970" t="n">
+        <v>0</v>
+      </c>
+      <c r="I1970" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1970" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1970" t="n">
+        <v>26.6</v>
+      </c>
+      <c r="L1970" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1971">
+      <c r="A1971" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B1971" t="inlineStr">
+        <is>
+          <t>1시</t>
+        </is>
+      </c>
+      <c r="C1971" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1971" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1971" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1971" t="n">
+        <v>25.7</v>
+      </c>
+      <c r="G1971" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="H1971" t="n">
+        <v>0</v>
+      </c>
+      <c r="I1971" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1971" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1971" t="n">
+        <v>25.7</v>
+      </c>
+      <c r="L1971" t="n">
+        <v>4.9</v>
+      </c>
+    </row>
+    <row r="1972">
+      <c r="A1972" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B1972" t="inlineStr">
+        <is>
+          <t>2시</t>
+        </is>
+      </c>
+      <c r="C1972" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1972" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1972" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1972" t="n">
+        <v>25</v>
+      </c>
+      <c r="G1972" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="H1972" t="n">
+        <v>0</v>
+      </c>
+      <c r="I1972" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1972" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1972" t="n">
+        <v>25</v>
+      </c>
+      <c r="L1972" t="n">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="1973">
+      <c r="A1973" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B1973" t="inlineStr">
+        <is>
+          <t>3시</t>
+        </is>
+      </c>
+      <c r="C1973" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1973" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1973" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1973" t="n">
+        <v>24.6</v>
+      </c>
+      <c r="G1973" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="H1973" t="n">
+        <v>0</v>
+      </c>
+      <c r="I1973" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1973" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1973" t="n">
+        <v>24.6</v>
+      </c>
+      <c r="L1973" t="n">
+        <v>2.7</v>
+      </c>
+    </row>
+    <row r="1974">
+      <c r="A1974" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B1974" t="inlineStr">
+        <is>
+          <t>4시</t>
+        </is>
+      </c>
+      <c r="C1974" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1974" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1974" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1974" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="G1974" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="H1974" t="n">
+        <v>0</v>
+      </c>
+      <c r="I1974" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1974" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1974" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="L1974" t="n">
+        <v>2.8</v>
+      </c>
+    </row>
+    <row r="1975">
+      <c r="A1975" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B1975" t="inlineStr">
+        <is>
+          <t>5시</t>
+        </is>
+      </c>
+      <c r="C1975" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1975" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1975" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1975" t="n">
+        <v>22.9</v>
+      </c>
+      <c r="G1975" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="H1975" t="n">
+        <v>0</v>
+      </c>
+      <c r="I1975" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1975" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1975" t="n">
+        <v>22.9</v>
+      </c>
+      <c r="L1975" t="n">
+        <v>3.2</v>
+      </c>
+    </row>
+    <row r="1976">
+      <c r="A1976" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B1976" t="inlineStr">
+        <is>
+          <t>6시</t>
+        </is>
+      </c>
+      <c r="C1976" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="D1976" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="E1976" t="n">
+        <v>5</v>
+      </c>
+      <c r="F1976" t="n">
+        <v>22.7</v>
+      </c>
+      <c r="G1976" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="H1976" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="I1976" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="J1976" t="n">
+        <v>5</v>
+      </c>
+      <c r="K1976" t="n">
+        <v>22.7</v>
+      </c>
+      <c r="L1976" t="n">
+        <v>2.9</v>
+      </c>
+    </row>
+    <row r="1977">
+      <c r="A1977" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B1977" t="inlineStr">
+        <is>
+          <t>7시</t>
+        </is>
+      </c>
+      <c r="C1977" t="n">
+        <v>8.710000000000001</v>
+      </c>
+      <c r="D1977" t="n">
+        <v>9.119999999999999</v>
+      </c>
+      <c r="E1977" t="n">
+        <v>108</v>
+      </c>
+      <c r="F1977" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="G1977" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="H1977" t="n">
+        <v>8.710000000000001</v>
+      </c>
+      <c r="I1977" t="n">
+        <v>9.119999999999999</v>
+      </c>
+      <c r="J1977" t="n">
+        <v>108</v>
+      </c>
+      <c r="K1977" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="L1977" t="n">
+        <v>4.1</v>
+      </c>
+    </row>
+    <row r="1978">
+      <c r="A1978" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B1978" t="inlineStr">
+        <is>
+          <t>8시</t>
+        </is>
+      </c>
+      <c r="C1978" t="n">
+        <v>23.21</v>
+      </c>
+      <c r="D1978" t="n">
+        <v>32.33</v>
+      </c>
+      <c r="E1978" t="n">
+        <v>297</v>
+      </c>
+      <c r="F1978" t="n">
+        <v>26.3</v>
+      </c>
+      <c r="G1978" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="H1978" t="n">
+        <v>23.21</v>
+      </c>
+      <c r="I1978" t="n">
+        <v>32.33</v>
+      </c>
+      <c r="J1978" t="n">
+        <v>297</v>
+      </c>
+      <c r="K1978" t="n">
+        <v>26.3</v>
+      </c>
+      <c r="L1978" t="n">
+        <v>6.6</v>
+      </c>
+    </row>
+    <row r="1979">
+      <c r="A1979" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B1979" t="inlineStr">
+        <is>
+          <t>9시</t>
+        </is>
+      </c>
+      <c r="C1979" t="n">
+        <v>37.08</v>
+      </c>
+      <c r="D1979" t="n">
+        <v>69.41</v>
+      </c>
+      <c r="E1979" t="n">
+        <v>492</v>
+      </c>
+      <c r="F1979" t="n">
+        <v>28.7</v>
+      </c>
+      <c r="G1979" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="H1979" t="n">
+        <v>37.08</v>
+      </c>
+      <c r="I1979" t="n">
+        <v>69.41</v>
+      </c>
+      <c r="J1979" t="n">
+        <v>492</v>
+      </c>
+      <c r="K1979" t="n">
+        <v>28.7</v>
+      </c>
+      <c r="L1979" t="n">
+        <v>8.1</v>
+      </c>
+    </row>
+    <row r="1980">
+      <c r="A1980" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B1980" t="inlineStr">
+        <is>
+          <t>10시</t>
+        </is>
+      </c>
+      <c r="C1980" t="n">
+        <v>49.31</v>
+      </c>
+      <c r="D1980" t="n">
+        <v>118.72</v>
+      </c>
+      <c r="E1980" t="n">
+        <v>675</v>
+      </c>
+      <c r="F1980" t="n">
+        <v>30.1</v>
+      </c>
+      <c r="G1980" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="H1980" t="n">
+        <v>49.31</v>
+      </c>
+      <c r="I1980" t="n">
+        <v>118.72</v>
+      </c>
+      <c r="J1980" t="n">
+        <v>675</v>
+      </c>
+      <c r="K1980" t="n">
+        <v>30.1</v>
+      </c>
+      <c r="L1980" t="n">
+        <v>8.6</v>
+      </c>
+    </row>
+    <row r="1981">
+      <c r="A1981" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B1981" t="inlineStr">
+        <is>
+          <t>11시</t>
+        </is>
+      </c>
+      <c r="C1981" t="n">
+        <v>58.21</v>
+      </c>
+      <c r="D1981" t="n">
+        <v>176.93</v>
+      </c>
+      <c r="E1981" t="n">
+        <v>820</v>
+      </c>
+      <c r="F1981" t="n">
+        <v>31.9</v>
+      </c>
+      <c r="G1981" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="H1981" t="n">
+        <v>58.21</v>
+      </c>
+      <c r="I1981" t="n">
+        <v>176.93</v>
+      </c>
+      <c r="J1981" t="n">
+        <v>820</v>
+      </c>
+      <c r="K1981" t="n">
+        <v>31.9</v>
+      </c>
+      <c r="L1981" t="n">
+        <v>9.4</v>
+      </c>
+    </row>
+    <row r="1982">
+      <c r="A1982" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B1982" t="inlineStr">
+        <is>
+          <t>12시</t>
+        </is>
+      </c>
+      <c r="C1982" t="n">
+        <v>63.5</v>
+      </c>
+      <c r="D1982" t="n">
+        <v>240.43</v>
+      </c>
+      <c r="E1982" t="n">
+        <v>913</v>
+      </c>
+      <c r="F1982" t="n">
+        <v>33.4</v>
+      </c>
+      <c r="G1982" t="n">
+        <v>10.6</v>
+      </c>
+      <c r="H1982" t="n">
+        <v>63.5</v>
+      </c>
+      <c r="I1982" t="n">
+        <v>240.43</v>
+      </c>
+      <c r="J1982" t="n">
+        <v>913</v>
+      </c>
+      <c r="K1982" t="n">
+        <v>33.4</v>
+      </c>
+      <c r="L1982" t="n">
+        <v>10.6</v>
+      </c>
+    </row>
+    <row r="1983">
+      <c r="A1983" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B1983" t="inlineStr">
+        <is>
+          <t>13시</t>
+        </is>
+      </c>
+      <c r="C1983" t="n">
+        <v>65.19</v>
+      </c>
+      <c r="D1983" t="n">
+        <v>305.62</v>
+      </c>
+      <c r="E1983" t="n">
+        <v>947</v>
+      </c>
+      <c r="F1983" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="G1983" t="n">
+        <v>11.6</v>
+      </c>
+      <c r="H1983" t="n">
+        <v>65.19</v>
+      </c>
+      <c r="I1983" t="n">
+        <v>305.62</v>
+      </c>
+      <c r="J1983" t="n">
+        <v>947</v>
+      </c>
+      <c r="K1983" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="L1983" t="n">
+        <v>11.6</v>
+      </c>
+    </row>
+    <row r="1984">
+      <c r="A1984" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B1984" t="inlineStr">
+        <is>
+          <t>14시</t>
+        </is>
+      </c>
+      <c r="C1984" t="n">
+        <v>63.29</v>
+      </c>
+      <c r="D1984" t="n">
+        <v>368.91</v>
+      </c>
+      <c r="E1984" t="n">
+        <v>919</v>
+      </c>
+      <c r="F1984" t="n">
+        <v>35.3</v>
+      </c>
+      <c r="G1984" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="H1984" t="n">
+        <v>63.29</v>
+      </c>
+      <c r="I1984" t="n">
+        <v>368.91</v>
+      </c>
+      <c r="J1984" t="n">
+        <v>919</v>
+      </c>
+      <c r="K1984" t="n">
+        <v>35.3</v>
+      </c>
+      <c r="L1984" t="n">
+        <v>14.2</v>
+      </c>
+    </row>
+    <row r="1985">
+      <c r="A1985" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B1985" t="inlineStr">
+        <is>
+          <t>15시</t>
+        </is>
+      </c>
+      <c r="C1985" t="n">
+        <v>57.84</v>
+      </c>
+      <c r="D1985" t="n">
+        <v>426.75</v>
+      </c>
+      <c r="E1985" t="n">
+        <v>832</v>
+      </c>
+      <c r="F1985" t="n">
+        <v>36</v>
+      </c>
+      <c r="G1985" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="H1985" t="n">
+        <v>57.84</v>
+      </c>
+      <c r="I1985" t="n">
+        <v>426.75</v>
+      </c>
+      <c r="J1985" t="n">
+        <v>832</v>
+      </c>
+      <c r="K1985" t="n">
+        <v>36</v>
+      </c>
+      <c r="L1985" t="n">
+        <v>11.5</v>
+      </c>
+    </row>
+    <row r="1986">
+      <c r="A1986" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B1986" t="inlineStr">
+        <is>
+          <t>16시</t>
+        </is>
+      </c>
+      <c r="C1986" t="n">
+        <v>49.43</v>
+      </c>
+      <c r="D1986" t="n">
+        <v>476.18</v>
+      </c>
+      <c r="E1986" t="n">
+        <v>694</v>
+      </c>
+      <c r="F1986" t="n">
+        <v>35.1</v>
+      </c>
+      <c r="G1986" t="n">
+        <v>16.6</v>
+      </c>
+      <c r="H1986" t="n">
+        <v>49.43</v>
+      </c>
+      <c r="I1986" t="n">
+        <v>476.18</v>
+      </c>
+      <c r="J1986" t="n">
+        <v>694</v>
+      </c>
+      <c r="K1986" t="n">
+        <v>35.1</v>
+      </c>
+      <c r="L1986" t="n">
+        <v>16.6</v>
+      </c>
+    </row>
+    <row r="1987">
+      <c r="A1987" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B1987" t="inlineStr">
+        <is>
+          <t>17시</t>
+        </is>
+      </c>
+      <c r="C1987" t="n">
+        <v>37.79</v>
+      </c>
+      <c r="D1987" t="n">
+        <v>513.97</v>
+      </c>
+      <c r="E1987" t="n">
+        <v>515</v>
+      </c>
+      <c r="F1987" t="n">
+        <v>34.1</v>
+      </c>
+      <c r="G1987" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="H1987" t="n">
+        <v>37.79</v>
+      </c>
+      <c r="I1987" t="n">
+        <v>513.97</v>
+      </c>
+      <c r="J1987" t="n">
+        <v>515</v>
+      </c>
+      <c r="K1987" t="n">
+        <v>34.1</v>
+      </c>
+      <c r="L1987" t="n">
+        <v>18.5</v>
+      </c>
+    </row>
+    <row r="1988">
+      <c r="A1988" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B1988" t="inlineStr">
+        <is>
+          <t>18시</t>
+        </is>
+      </c>
+      <c r="C1988" t="n">
+        <v>24.01</v>
+      </c>
+      <c r="D1988" t="n">
+        <v>537.98</v>
+      </c>
+      <c r="E1988" t="n">
+        <v>317</v>
+      </c>
+      <c r="F1988" t="n">
+        <v>33</v>
+      </c>
+      <c r="G1988" t="n">
+        <v>15.6</v>
+      </c>
+      <c r="H1988" t="n">
+        <v>24.01</v>
+      </c>
+      <c r="I1988" t="n">
+        <v>537.98</v>
+      </c>
+      <c r="J1988" t="n">
+        <v>317</v>
+      </c>
+      <c r="K1988" t="n">
+        <v>33</v>
+      </c>
+      <c r="L1988" t="n">
+        <v>15.6</v>
+      </c>
+    </row>
+    <row r="1989">
+      <c r="A1989" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B1989" t="inlineStr">
+        <is>
+          <t>19시</t>
+        </is>
+      </c>
+      <c r="C1989" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="D1989" t="n">
+        <v>548.28</v>
+      </c>
+      <c r="E1989" t="n">
+        <v>132</v>
+      </c>
+      <c r="F1989" t="n">
+        <v>31.7</v>
+      </c>
+      <c r="G1989" t="n">
+        <v>10.9</v>
+      </c>
+      <c r="H1989" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="I1989" t="n">
+        <v>548.28</v>
+      </c>
+      <c r="J1989" t="n">
+        <v>132</v>
+      </c>
+      <c r="K1989" t="n">
+        <v>31.7</v>
+      </c>
+      <c r="L1989" t="n">
+        <v>10.9</v>
+      </c>
+    </row>
+    <row r="1990">
+      <c r="A1990" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B1990" t="inlineStr">
+        <is>
+          <t>20시</t>
+        </is>
+      </c>
+      <c r="C1990" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="D1990" t="n">
+        <v>549.08</v>
+      </c>
+      <c r="E1990" t="n">
+        <v>10</v>
+      </c>
+      <c r="F1990" t="n">
+        <v>30</v>
+      </c>
+      <c r="G1990" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="H1990" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="I1990" t="n">
+        <v>549.08</v>
+      </c>
+      <c r="J1990" t="n">
+        <v>10</v>
+      </c>
+      <c r="K1990" t="n">
+        <v>30</v>
+      </c>
+      <c r="L1990" t="n">
+        <v>7.3</v>
+      </c>
+    </row>
+    <row r="1991">
+      <c r="A1991" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B1991" t="inlineStr">
+        <is>
+          <t>21시</t>
+        </is>
+      </c>
+      <c r="C1991" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1991" t="n">
+        <v>549.08</v>
+      </c>
+      <c r="E1991" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1991" t="n">
+        <v>28.8</v>
+      </c>
+      <c r="G1991" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="H1991" t="n">
+        <v>0</v>
+      </c>
+      <c r="I1991" t="n">
+        <v>549.08</v>
+      </c>
+      <c r="J1991" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1991" t="n">
+        <v>28.8</v>
+      </c>
+      <c r="L1991" t="n">
+        <v>4.6</v>
+      </c>
+    </row>
+    <row r="1992">
+      <c r="A1992" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B1992" t="inlineStr">
+        <is>
+          <t>22시</t>
+        </is>
+      </c>
+      <c r="C1992" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1992" t="n">
+        <v>549.08</v>
+      </c>
+      <c r="E1992" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1992" t="n">
+        <v>27.9</v>
+      </c>
+      <c r="G1992" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="H1992" t="n">
+        <v>0</v>
+      </c>
+      <c r="I1992" t="n">
+        <v>549.08</v>
+      </c>
+      <c r="J1992" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1992" t="n">
+        <v>27.9</v>
+      </c>
+      <c r="L1992" t="n">
+        <v>4.8</v>
+      </c>
+    </row>
+    <row r="1993">
+      <c r="A1993" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B1993" t="inlineStr">
+        <is>
+          <t>23시</t>
+        </is>
+      </c>
+      <c r="C1993" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1993" t="n">
+        <v>549.08</v>
+      </c>
+      <c r="E1993" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1993" t="n">
+        <v>27</v>
+      </c>
+      <c r="G1993" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="H1993" t="n">
+        <v>0</v>
+      </c>
+      <c r="I1993" t="n">
+        <v>549.08</v>
+      </c>
+      <c r="J1993" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1993" t="n">
+        <v>27</v>
+      </c>
+      <c r="L1993" t="n">
+        <v>4.4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto: solar data update 2026-08-01
</commit_message>
<xml_diff>
--- a/log.xlsx
+++ b/log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1993"/>
+  <dimension ref="A1:L2017"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -84622,6 +84622,1014 @@
         <v>4.4</v>
       </c>
     </row>
+    <row r="1994">
+      <c r="A1994" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B1994" t="inlineStr">
+        <is>
+          <t>0시</t>
+        </is>
+      </c>
+      <c r="C1994" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1994" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1994" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1994" t="n">
+        <v>26</v>
+      </c>
+      <c r="G1994" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="H1994" t="n">
+        <v>0</v>
+      </c>
+      <c r="I1994" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1994" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1994" t="n">
+        <v>26</v>
+      </c>
+      <c r="L1994" t="n">
+        <v>4.8</v>
+      </c>
+    </row>
+    <row r="1995">
+      <c r="A1995" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B1995" t="inlineStr">
+        <is>
+          <t>1시</t>
+        </is>
+      </c>
+      <c r="C1995" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1995" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1995" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1995" t="n">
+        <v>25.3</v>
+      </c>
+      <c r="G1995" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="H1995" t="n">
+        <v>0</v>
+      </c>
+      <c r="I1995" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1995" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1995" t="n">
+        <v>25.3</v>
+      </c>
+      <c r="L1995" t="n">
+        <v>4.2</v>
+      </c>
+    </row>
+    <row r="1996">
+      <c r="A1996" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B1996" t="inlineStr">
+        <is>
+          <t>2시</t>
+        </is>
+      </c>
+      <c r="C1996" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1996" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1996" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1996" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="G1996" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="H1996" t="n">
+        <v>0</v>
+      </c>
+      <c r="I1996" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1996" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1996" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="L1996" t="n">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="1997">
+      <c r="A1997" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B1997" t="inlineStr">
+        <is>
+          <t>3시</t>
+        </is>
+      </c>
+      <c r="C1997" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1997" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1997" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1997" t="n">
+        <v>24.3</v>
+      </c>
+      <c r="G1997" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="H1997" t="n">
+        <v>0</v>
+      </c>
+      <c r="I1997" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1997" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1997" t="n">
+        <v>24.3</v>
+      </c>
+      <c r="L1997" t="n">
+        <v>3.7</v>
+      </c>
+    </row>
+    <row r="1998">
+      <c r="A1998" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B1998" t="inlineStr">
+        <is>
+          <t>4시</t>
+        </is>
+      </c>
+      <c r="C1998" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1998" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1998" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1998" t="n">
+        <v>23.4</v>
+      </c>
+      <c r="G1998" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="H1998" t="n">
+        <v>0</v>
+      </c>
+      <c r="I1998" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1998" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1998" t="n">
+        <v>23.4</v>
+      </c>
+      <c r="L1998" t="n">
+        <v>3.4</v>
+      </c>
+    </row>
+    <row r="1999">
+      <c r="A1999" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B1999" t="inlineStr">
+        <is>
+          <t>5시</t>
+        </is>
+      </c>
+      <c r="C1999" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1999" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1999" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1999" t="n">
+        <v>22.9</v>
+      </c>
+      <c r="G1999" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="H1999" t="n">
+        <v>0</v>
+      </c>
+      <c r="I1999" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1999" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1999" t="n">
+        <v>22.9</v>
+      </c>
+      <c r="L1999" t="n">
+        <v>2.7</v>
+      </c>
+    </row>
+    <row r="2000">
+      <c r="A2000" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B2000" t="inlineStr">
+        <is>
+          <t>6시</t>
+        </is>
+      </c>
+      <c r="C2000" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="D2000" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="E2000" t="n">
+        <v>4</v>
+      </c>
+      <c r="F2000" t="n">
+        <v>22.7</v>
+      </c>
+      <c r="G2000" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="H2000" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="I2000" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="J2000" t="n">
+        <v>4</v>
+      </c>
+      <c r="K2000" t="n">
+        <v>22.7</v>
+      </c>
+      <c r="L2000" t="n">
+        <v>2.6</v>
+      </c>
+    </row>
+    <row r="2001">
+      <c r="A2001" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B2001" t="inlineStr">
+        <is>
+          <t>7시</t>
+        </is>
+      </c>
+      <c r="C2001" t="n">
+        <v>8.470000000000001</v>
+      </c>
+      <c r="D2001" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="E2001" t="n">
+        <v>105</v>
+      </c>
+      <c r="F2001" t="n">
+        <v>24.7</v>
+      </c>
+      <c r="G2001" t="n">
+        <v>4</v>
+      </c>
+      <c r="H2001" t="n">
+        <v>8.470000000000001</v>
+      </c>
+      <c r="I2001" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="J2001" t="n">
+        <v>105</v>
+      </c>
+      <c r="K2001" t="n">
+        <v>24.7</v>
+      </c>
+      <c r="L2001" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2002">
+      <c r="A2002" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B2002" t="inlineStr">
+        <is>
+          <t>8시</t>
+        </is>
+      </c>
+      <c r="C2002" t="n">
+        <v>22.96</v>
+      </c>
+      <c r="D2002" t="n">
+        <v>31.76</v>
+      </c>
+      <c r="E2002" t="n">
+        <v>294</v>
+      </c>
+      <c r="F2002" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="G2002" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="H2002" t="n">
+        <v>22.96</v>
+      </c>
+      <c r="I2002" t="n">
+        <v>31.76</v>
+      </c>
+      <c r="J2002" t="n">
+        <v>294</v>
+      </c>
+      <c r="K2002" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="L2002" t="n">
+        <v>5.3</v>
+      </c>
+    </row>
+    <row r="2003">
+      <c r="A2003" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B2003" t="inlineStr">
+        <is>
+          <t>9시</t>
+        </is>
+      </c>
+      <c r="C2003" t="n">
+        <v>37.27</v>
+      </c>
+      <c r="D2003" t="n">
+        <v>69.03</v>
+      </c>
+      <c r="E2003" t="n">
+        <v>496</v>
+      </c>
+      <c r="F2003" t="n">
+        <v>29.3</v>
+      </c>
+      <c r="G2003" t="n">
+        <v>7</v>
+      </c>
+      <c r="H2003" t="n">
+        <v>37.27</v>
+      </c>
+      <c r="I2003" t="n">
+        <v>69.03</v>
+      </c>
+      <c r="J2003" t="n">
+        <v>496</v>
+      </c>
+      <c r="K2003" t="n">
+        <v>29.3</v>
+      </c>
+      <c r="L2003" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2004">
+      <c r="A2004" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B2004" t="inlineStr">
+        <is>
+          <t>10시</t>
+        </is>
+      </c>
+      <c r="C2004" t="n">
+        <v>49.07</v>
+      </c>
+      <c r="D2004" t="n">
+        <v>118.1</v>
+      </c>
+      <c r="E2004" t="n">
+        <v>675</v>
+      </c>
+      <c r="F2004" t="n">
+        <v>31.2</v>
+      </c>
+      <c r="G2004" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="H2004" t="n">
+        <v>49.07</v>
+      </c>
+      <c r="I2004" t="n">
+        <v>118.1</v>
+      </c>
+      <c r="J2004" t="n">
+        <v>675</v>
+      </c>
+      <c r="K2004" t="n">
+        <v>31.2</v>
+      </c>
+      <c r="L2004" t="n">
+        <v>5.8</v>
+      </c>
+    </row>
+    <row r="2005">
+      <c r="A2005" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B2005" t="inlineStr">
+        <is>
+          <t>11시</t>
+        </is>
+      </c>
+      <c r="C2005" t="n">
+        <v>57.49</v>
+      </c>
+      <c r="D2005" t="n">
+        <v>175.59</v>
+      </c>
+      <c r="E2005" t="n">
+        <v>815</v>
+      </c>
+      <c r="F2005" t="n">
+        <v>33.4</v>
+      </c>
+      <c r="G2005" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="H2005" t="n">
+        <v>57.49</v>
+      </c>
+      <c r="I2005" t="n">
+        <v>175.59</v>
+      </c>
+      <c r="J2005" t="n">
+        <v>815</v>
+      </c>
+      <c r="K2005" t="n">
+        <v>33.4</v>
+      </c>
+      <c r="L2005" t="n">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="2006">
+      <c r="A2006" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B2006" t="inlineStr">
+        <is>
+          <t>12시</t>
+        </is>
+      </c>
+      <c r="C2006" t="n">
+        <v>62.63</v>
+      </c>
+      <c r="D2006" t="n">
+        <v>238.22</v>
+      </c>
+      <c r="E2006" t="n">
+        <v>906</v>
+      </c>
+      <c r="F2006" t="n">
+        <v>34.9</v>
+      </c>
+      <c r="G2006" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="H2006" t="n">
+        <v>62.63</v>
+      </c>
+      <c r="I2006" t="n">
+        <v>238.22</v>
+      </c>
+      <c r="J2006" t="n">
+        <v>906</v>
+      </c>
+      <c r="K2006" t="n">
+        <v>34.9</v>
+      </c>
+      <c r="L2006" t="n">
+        <v>5.6</v>
+      </c>
+    </row>
+    <row r="2007">
+      <c r="A2007" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B2007" t="inlineStr">
+        <is>
+          <t>13시</t>
+        </is>
+      </c>
+      <c r="C2007" t="n">
+        <v>64.23</v>
+      </c>
+      <c r="D2007" t="n">
+        <v>302.45</v>
+      </c>
+      <c r="E2007" t="n">
+        <v>938</v>
+      </c>
+      <c r="F2007" t="n">
+        <v>35.9</v>
+      </c>
+      <c r="G2007" t="n">
+        <v>6</v>
+      </c>
+      <c r="H2007" t="n">
+        <v>64.23</v>
+      </c>
+      <c r="I2007" t="n">
+        <v>302.45</v>
+      </c>
+      <c r="J2007" t="n">
+        <v>938</v>
+      </c>
+      <c r="K2007" t="n">
+        <v>35.9</v>
+      </c>
+      <c r="L2007" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2008">
+      <c r="A2008" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B2008" t="inlineStr">
+        <is>
+          <t>14시</t>
+        </is>
+      </c>
+      <c r="C2008" t="n">
+        <v>62.27</v>
+      </c>
+      <c r="D2008" t="n">
+        <v>364.72</v>
+      </c>
+      <c r="E2008" t="n">
+        <v>910</v>
+      </c>
+      <c r="F2008" t="n">
+        <v>36.9</v>
+      </c>
+      <c r="G2008" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="H2008" t="n">
+        <v>62.27</v>
+      </c>
+      <c r="I2008" t="n">
+        <v>364.72</v>
+      </c>
+      <c r="J2008" t="n">
+        <v>910</v>
+      </c>
+      <c r="K2008" t="n">
+        <v>36.9</v>
+      </c>
+      <c r="L2008" t="n">
+        <v>6.3</v>
+      </c>
+    </row>
+    <row r="2009">
+      <c r="A2009" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B2009" t="inlineStr">
+        <is>
+          <t>15시</t>
+        </is>
+      </c>
+      <c r="C2009" t="n">
+        <v>56.51</v>
+      </c>
+      <c r="D2009" t="n">
+        <v>421.23</v>
+      </c>
+      <c r="E2009" t="n">
+        <v>819</v>
+      </c>
+      <c r="F2009" t="n">
+        <v>38</v>
+      </c>
+      <c r="G2009" t="n">
+        <v>9.699999999999999</v>
+      </c>
+      <c r="H2009" t="n">
+        <v>56.51</v>
+      </c>
+      <c r="I2009" t="n">
+        <v>421.23</v>
+      </c>
+      <c r="J2009" t="n">
+        <v>819</v>
+      </c>
+      <c r="K2009" t="n">
+        <v>38</v>
+      </c>
+      <c r="L2009" t="n">
+        <v>9.699999999999999</v>
+      </c>
+    </row>
+    <row r="2010">
+      <c r="A2010" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B2010" t="inlineStr">
+        <is>
+          <t>16시</t>
+        </is>
+      </c>
+      <c r="C2010" t="n">
+        <v>46.91</v>
+      </c>
+      <c r="D2010" t="n">
+        <v>468.14</v>
+      </c>
+      <c r="E2010" t="n">
+        <v>663</v>
+      </c>
+      <c r="F2010" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="G2010" t="n">
+        <v>10.6</v>
+      </c>
+      <c r="H2010" t="n">
+        <v>46.91</v>
+      </c>
+      <c r="I2010" t="n">
+        <v>468.14</v>
+      </c>
+      <c r="J2010" t="n">
+        <v>663</v>
+      </c>
+      <c r="K2010" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="L2010" t="n">
+        <v>10.6</v>
+      </c>
+    </row>
+    <row r="2011">
+      <c r="A2011" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B2011" t="inlineStr">
+        <is>
+          <t>17시</t>
+        </is>
+      </c>
+      <c r="C2011" t="n">
+        <v>36.22</v>
+      </c>
+      <c r="D2011" t="n">
+        <v>504.36</v>
+      </c>
+      <c r="E2011" t="n">
+        <v>499</v>
+      </c>
+      <c r="F2011" t="n">
+        <v>37</v>
+      </c>
+      <c r="G2011" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="H2011" t="n">
+        <v>36.22</v>
+      </c>
+      <c r="I2011" t="n">
+        <v>504.36</v>
+      </c>
+      <c r="J2011" t="n">
+        <v>499</v>
+      </c>
+      <c r="K2011" t="n">
+        <v>37</v>
+      </c>
+      <c r="L2011" t="n">
+        <v>13.5</v>
+      </c>
+    </row>
+    <row r="2012">
+      <c r="A2012" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B2012" t="inlineStr">
+        <is>
+          <t>18시</t>
+        </is>
+      </c>
+      <c r="C2012" t="n">
+        <v>22.67</v>
+      </c>
+      <c r="D2012" t="n">
+        <v>527.03</v>
+      </c>
+      <c r="E2012" t="n">
+        <v>302</v>
+      </c>
+      <c r="F2012" t="n">
+        <v>35.6</v>
+      </c>
+      <c r="G2012" t="n">
+        <v>17.1</v>
+      </c>
+      <c r="H2012" t="n">
+        <v>22.67</v>
+      </c>
+      <c r="I2012" t="n">
+        <v>527.03</v>
+      </c>
+      <c r="J2012" t="n">
+        <v>302</v>
+      </c>
+      <c r="K2012" t="n">
+        <v>35.6</v>
+      </c>
+      <c r="L2012" t="n">
+        <v>17.1</v>
+      </c>
+    </row>
+    <row r="2013">
+      <c r="A2013" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B2013" t="inlineStr">
+        <is>
+          <t>19시</t>
+        </is>
+      </c>
+      <c r="C2013" t="n">
+        <v>9.68</v>
+      </c>
+      <c r="D2013" t="n">
+        <v>536.71</v>
+      </c>
+      <c r="E2013" t="n">
+        <v>125</v>
+      </c>
+      <c r="F2013" t="n">
+        <v>33.8</v>
+      </c>
+      <c r="G2013" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="H2013" t="n">
+        <v>9.68</v>
+      </c>
+      <c r="I2013" t="n">
+        <v>536.71</v>
+      </c>
+      <c r="J2013" t="n">
+        <v>125</v>
+      </c>
+      <c r="K2013" t="n">
+        <v>33.8</v>
+      </c>
+      <c r="L2013" t="n">
+        <v>16.9</v>
+      </c>
+    </row>
+    <row r="2014">
+      <c r="A2014" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B2014" t="inlineStr">
+        <is>
+          <t>20시</t>
+        </is>
+      </c>
+      <c r="C2014" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="D2014" t="n">
+        <v>537.42</v>
+      </c>
+      <c r="E2014" t="n">
+        <v>9</v>
+      </c>
+      <c r="F2014" t="n">
+        <v>32</v>
+      </c>
+      <c r="G2014" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="H2014" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="I2014" t="n">
+        <v>537.42</v>
+      </c>
+      <c r="J2014" t="n">
+        <v>9</v>
+      </c>
+      <c r="K2014" t="n">
+        <v>32</v>
+      </c>
+      <c r="L2014" t="n">
+        <v>10.7</v>
+      </c>
+    </row>
+    <row r="2015">
+      <c r="A2015" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B2015" t="inlineStr">
+        <is>
+          <t>21시</t>
+        </is>
+      </c>
+      <c r="C2015" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2015" t="n">
+        <v>537.42</v>
+      </c>
+      <c r="E2015" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2015" t="n">
+        <v>30.8</v>
+      </c>
+      <c r="G2015" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="H2015" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2015" t="n">
+        <v>537.42</v>
+      </c>
+      <c r="J2015" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2015" t="n">
+        <v>30.8</v>
+      </c>
+      <c r="L2015" t="n">
+        <v>6.8</v>
+      </c>
+    </row>
+    <row r="2016">
+      <c r="A2016" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B2016" t="inlineStr">
+        <is>
+          <t>22시</t>
+        </is>
+      </c>
+      <c r="C2016" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2016" t="n">
+        <v>537.42</v>
+      </c>
+      <c r="E2016" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2016" t="n">
+        <v>29.8</v>
+      </c>
+      <c r="G2016" t="n">
+        <v>5</v>
+      </c>
+      <c r="H2016" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2016" t="n">
+        <v>537.42</v>
+      </c>
+      <c r="J2016" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2016" t="n">
+        <v>29.8</v>
+      </c>
+      <c r="L2016" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2017">
+      <c r="A2017" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B2017" t="inlineStr">
+        <is>
+          <t>23시</t>
+        </is>
+      </c>
+      <c r="C2017" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2017" t="n">
+        <v>537.42</v>
+      </c>
+      <c r="E2017" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2017" t="n">
+        <v>28.7</v>
+      </c>
+      <c r="G2017" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="H2017" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2017" t="n">
+        <v>537.42</v>
+      </c>
+      <c r="J2017" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2017" t="n">
+        <v>28.7</v>
+      </c>
+      <c r="L2017" t="n">
+        <v>4.8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>